<commit_message>
Inclusão de script vinculo de ordem em massa
</commit_message>
<xml_diff>
--- a/Planilhas/Imobilizados_AS01.xlsx
+++ b/Planilhas/Imobilizados_AS01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python_scripts\Planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1897F5AA-DDBA-4A1C-A538-CCFE9D958D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D64812D-DD3A-4B59-915C-DBD3F10FADFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28635" yWindow="-135" windowWidth="29130" windowHeight="15810" xr2:uid="{F747952C-0BBF-40FF-A04B-44C1B13F3EC3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="27">
   <si>
     <t>Denominação</t>
   </si>
@@ -74,95 +74,56 @@
     <t>Ordem</t>
   </si>
   <si>
-    <t>SWITCH CISCO BUSINESS 220 24 PORTAS</t>
+    <t>AR CONDICIONADO SPLIT</t>
   </si>
   <si>
-    <t>20011AD028</t>
+    <t>CONDESADORA SPLIT-INVERTER</t>
   </si>
   <si>
-    <t>600017</t>
+    <t>CADEIRA DIRETOR</t>
   </si>
   <si>
-    <t>SWITCH CISCO BUSINESS 220 24 PORTAS  POE LAYER 2</t>
+    <t>DEA-DESFIBRILADOR LIFE</t>
   </si>
   <si>
-    <t xml:space="preserve">DNI27230121              </t>
+    <t>CADEIRA GIRATORIA CAVALETTI</t>
   </si>
   <si>
-    <t xml:space="preserve">DNI272006ZZ              </t>
+    <t>MESA CAFE</t>
   </si>
   <si>
-    <t xml:space="preserve">DNI2723014L              </t>
+    <t>ARMARIO COM ARQUIVO 04 PASTAS COM NICHO</t>
   </si>
   <si>
-    <t xml:space="preserve">DNI2823005E              </t>
+    <t>ARMARIO MEDIO 02 PORTAS PADRAO CF</t>
   </si>
   <si>
-    <t xml:space="preserve">DNI2823005V              </t>
+    <t>MESA DE REUNIAO 1600/2000MM PADRAO CF</t>
   </si>
   <si>
-    <t xml:space="preserve">DNI27230DLZ              </t>
+    <t>MESA PE PAINEL1,20M MDF 2 LUGARES</t>
   </si>
   <si>
-    <t xml:space="preserve">DNI27200705              </t>
+    <t>CALL CENTER 25MM 15MM 950X680X1150MM</t>
   </si>
   <si>
-    <t xml:space="preserve">DNI27230125              </t>
+    <t>CALL CENTER 25MM ACP 925X680X1150MM</t>
   </si>
   <si>
-    <t xml:space="preserve">DNI2723012B              </t>
+    <t>20011PI035</t>
   </si>
   <si>
-    <t xml:space="preserve">DNI2723014B              </t>
+    <t>20011AD020</t>
   </si>
   <si>
-    <t xml:space="preserve">DNI2823006J              </t>
-  </si>
-  <si>
-    <t xml:space="preserve">DNI2823004W              </t>
-  </si>
-  <si>
-    <t xml:space="preserve">DNI27230DJ1              </t>
-  </si>
-  <si>
-    <t xml:space="preserve">DNI2723012P              </t>
-  </si>
-  <si>
-    <t xml:space="preserve">DNI2723014N              </t>
-  </si>
-  <si>
-    <t xml:space="preserve">DNI27230DN0              </t>
-  </si>
-  <si>
-    <t xml:space="preserve">DNI27230DHD              </t>
-  </si>
-  <si>
-    <t xml:space="preserve">DNI2723011H              </t>
-  </si>
-  <si>
-    <t>NOBREAK 8KVA 220V/220V</t>
-  </si>
-  <si>
-    <t>SWITCH CISCO C1300-24XS 24-PORTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WZP28289X0N              </t>
-  </si>
-  <si>
-    <t xml:space="preserve">WZP28289M3F              </t>
-  </si>
-  <si>
-    <t>SWITCH CISCO BUSINESS 220</t>
-  </si>
-  <si>
-    <t>SWITCH CISCO C1300 - 24XS - CATALYST</t>
+    <t>600023</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -172,6 +133,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -258,7 +226,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -268,29 +236,13 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="16">
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -366,8 +318,6 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -381,6 +331,75 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
@@ -406,24 +425,8 @@
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -510,42 +513,6 @@
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color indexed="64"/>
@@ -601,21 +568,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E1A2811A-4DE7-4797-909B-034865ED5825}" name="Tabela1" displayName="Tabela1" ref="A1:L63" totalsRowShown="0" headerRowDxfId="15" headerRowBorderDxfId="14" tableBorderDxfId="13" totalsRowBorderDxfId="12">
-  <autoFilter ref="A1:L63" xr:uid="{E1A2811A-4DE7-4797-909B-034865ED5825}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E1A2811A-4DE7-4797-909B-034865ED5825}" name="Tabela1" displayName="Tabela1" ref="A1:L65" totalsRowShown="0" headerRowDxfId="15" headerRowBorderDxfId="14" tableBorderDxfId="13" totalsRowBorderDxfId="12">
+  <autoFilter ref="A1:L65" xr:uid="{E1A2811A-4DE7-4797-909B-034865ED5825}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{9308F4FF-4ADE-4BF4-88E4-470CF2104708}" name="Classe" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{F2468D06-3D0A-4294-9CD8-5504956F01F9}" name="Denominação" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{A201AFA3-7F35-41FE-861A-ACB6C97DC90A}" name="Serie" dataDxfId="9"/>
-    <tableColumn id="11" xr3:uid="{BEB32E32-BA86-47E9-8D5D-2275177A4999}" name="Inventario" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{B8D2BEFF-D66E-4518-B857-1D984936B5C7}" name="Centro de custo" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{8549FA69-682D-4B77-9716-42E5D1100582}" name="Centro" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{18501CF4-B734-437A-A00B-B431A493C777}" name="Criterio_1" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{9EAD43B9-ACF0-4216-AFF2-BCCA28D73236}" name="Criterio_2" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{0C188A2F-C5F0-4980-B0CF-7AF60D5F1B38}" name="Ordem" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{02EAF220-4016-4DFA-96A6-D870D7A47E92}" name="Vida" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{E08E8965-3965-422A-ADDC-8101963314B9}" name="Depreciação" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{9497B329-73F9-4A84-B10F-4A000E710F4F}" name="Depreciação_Fiscal" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{9308F4FF-4ADE-4BF4-88E4-470CF2104708}" name="Classe" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{F2468D06-3D0A-4294-9CD8-5504956F01F9}" name="Denominação" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{A201AFA3-7F35-41FE-861A-ACB6C97DC90A}" name="Serie" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{BEB32E32-BA86-47E9-8D5D-2275177A4999}" name="Inventario" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{B8D2BEFF-D66E-4518-B857-1D984936B5C7}" name="Centro de custo" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{8549FA69-682D-4B77-9716-42E5D1100582}" name="Centro" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{18501CF4-B734-437A-A00B-B431A493C777}" name="Criterio_1" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{9EAD43B9-ACF0-4216-AFF2-BCCA28D73236}" name="Criterio_2" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{0C188A2F-C5F0-4980-B0CF-7AF60D5F1B38}" name="Ordem" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{02EAF220-4016-4DFA-96A6-D870D7A47E92}" name="Vida" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{E08E8965-3965-422A-ADDC-8101963314B9}" name="Depreciação" dataDxfId="0"/>
+    <tableColumn id="9" xr3:uid="{9497B329-73F9-4A84-B10F-4A000E710F4F}" name="Depreciação_Fiscal" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -938,7 +905,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF4B497B-760A-4B7F-8915-5B5F35428092}">
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="71" bestFit="1" customWidth="1"/>
@@ -993,19 +960,15 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="5">
-        <v>18674</v>
-      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
       <c r="E2" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F2" s="5">
         <v>2001</v>
@@ -1013,12 +976,12 @@
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
       <c r="I2" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J2" s="5">
-        <v>10</v>
-      </c>
-      <c r="K2" s="7">
+        <v>15</v>
+      </c>
+      <c r="K2" s="8">
         <v>46113</v>
       </c>
       <c r="L2" s="4">
@@ -1027,19 +990,15 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="5">
-        <v>18675</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
       <c r="E3" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F3" s="5">
         <v>2001</v>
@@ -1047,12 +1006,12 @@
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
       <c r="I3" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J3" s="5">
-        <v>10</v>
-      </c>
-      <c r="K3" s="7">
+        <v>15</v>
+      </c>
+      <c r="K3" s="8">
         <v>46113</v>
       </c>
       <c r="L3" s="4">
@@ -1061,19 +1020,15 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="5">
-        <v>18676</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
       <c r="E4" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F4" s="5">
         <v>2001</v>
@@ -1081,12 +1036,12 @@
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
       <c r="I4" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J4" s="5">
-        <v>10</v>
-      </c>
-      <c r="K4" s="7">
+        <v>15</v>
+      </c>
+      <c r="K4" s="8">
         <v>46113</v>
       </c>
       <c r="L4" s="4">
@@ -1095,19 +1050,15 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="5">
-        <v>18677</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
       <c r="E5" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F5" s="5">
         <v>2001</v>
@@ -1115,12 +1066,12 @@
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
       <c r="I5" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J5" s="5">
-        <v>10</v>
-      </c>
-      <c r="K5" s="7">
+        <v>15</v>
+      </c>
+      <c r="K5" s="8">
         <v>46113</v>
       </c>
       <c r="L5" s="4">
@@ -1129,19 +1080,15 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="5">
-        <v>18678</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F6" s="5">
         <v>2001</v>
@@ -1149,12 +1096,12 @@
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
       <c r="I6" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J6" s="5">
-        <v>10</v>
-      </c>
-      <c r="K6" s="7">
+        <v>15</v>
+      </c>
+      <c r="K6" s="8">
         <v>46113</v>
       </c>
       <c r="L6" s="4">
@@ -1163,19 +1110,15 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="5">
-        <v>18679</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
       <c r="E7" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F7" s="5">
         <v>2001</v>
@@ -1183,12 +1126,12 @@
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
       <c r="I7" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J7" s="5">
-        <v>10</v>
-      </c>
-      <c r="K7" s="7">
+        <v>15</v>
+      </c>
+      <c r="K7" s="8">
         <v>46113</v>
       </c>
       <c r="L7" s="4">
@@ -1197,19 +1140,15 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="5">
-        <v>18680</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
       <c r="E8" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F8" s="5">
         <v>2001</v>
@@ -1217,12 +1156,12 @@
       <c r="G8" s="5"/>
       <c r="H8" s="5"/>
       <c r="I8" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J8" s="5">
-        <v>10</v>
-      </c>
-      <c r="K8" s="7">
+        <v>15</v>
+      </c>
+      <c r="K8" s="8">
         <v>46113</v>
       </c>
       <c r="L8" s="4">
@@ -1231,19 +1170,15 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" s="5">
-        <v>18681</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
       <c r="E9" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F9" s="5">
         <v>2001</v>
@@ -1251,12 +1186,12 @@
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
       <c r="I9" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J9" s="5">
-        <v>10</v>
-      </c>
-      <c r="K9" s="7">
+        <v>15</v>
+      </c>
+      <c r="K9" s="8">
         <v>46113</v>
       </c>
       <c r="L9" s="4">
@@ -1265,19 +1200,15 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D10" s="5">
-        <v>18682</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
       <c r="E10" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F10" s="5">
         <v>2001</v>
@@ -1285,12 +1216,12 @@
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
       <c r="I10" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J10" s="5">
-        <v>10</v>
-      </c>
-      <c r="K10" s="7">
+        <v>15</v>
+      </c>
+      <c r="K10" s="8">
         <v>46113</v>
       </c>
       <c r="L10" s="4">
@@ -1299,19 +1230,15 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" s="5">
-        <v>18683</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
       <c r="E11" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F11" s="5">
         <v>2001</v>
@@ -1319,12 +1246,12 @@
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
       <c r="I11" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J11" s="5">
-        <v>10</v>
-      </c>
-      <c r="K11" s="7">
+        <v>15</v>
+      </c>
+      <c r="K11" s="8">
         <v>46113</v>
       </c>
       <c r="L11" s="4">
@@ -1333,19 +1260,15 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D12" s="5">
-        <v>18684</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
       <c r="E12" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F12" s="5">
         <v>2001</v>
@@ -1353,12 +1276,12 @@
       <c r="G12" s="5"/>
       <c r="H12" s="5"/>
       <c r="I12" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J12" s="5">
-        <v>10</v>
-      </c>
-      <c r="K12" s="7">
+        <v>15</v>
+      </c>
+      <c r="K12" s="8">
         <v>46113</v>
       </c>
       <c r="L12" s="4">
@@ -1367,19 +1290,15 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="5">
-        <v>18685</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
       <c r="E13" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F13" s="5">
         <v>2001</v>
@@ -1387,12 +1306,12 @@
       <c r="G13" s="5"/>
       <c r="H13" s="5"/>
       <c r="I13" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J13" s="5">
-        <v>10</v>
-      </c>
-      <c r="K13" s="7">
+        <v>15</v>
+      </c>
+      <c r="K13" s="8">
         <v>46113</v>
       </c>
       <c r="L13" s="4">
@@ -1401,19 +1320,15 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" s="5">
-        <v>18686</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
       <c r="E14" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F14" s="5">
         <v>2001</v>
@@ -1421,12 +1336,12 @@
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
       <c r="I14" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J14" s="5">
-        <v>10</v>
-      </c>
-      <c r="K14" s="7">
+        <v>15</v>
+      </c>
+      <c r="K14" s="8">
         <v>46113</v>
       </c>
       <c r="L14" s="4">
@@ -1435,19 +1350,15 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D15" s="5">
-        <v>18687</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
       <c r="E15" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F15" s="5">
         <v>2001</v>
@@ -1455,12 +1366,12 @@
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
       <c r="I15" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J15" s="5">
-        <v>10</v>
-      </c>
-      <c r="K15" s="7">
+        <v>15</v>
+      </c>
+      <c r="K15" s="8">
         <v>46113</v>
       </c>
       <c r="L15" s="4">
@@ -1469,19 +1380,15 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D16" s="5">
-        <v>18688</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
       <c r="E16" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F16" s="5">
         <v>2001</v>
@@ -1489,12 +1396,12 @@
       <c r="G16" s="5"/>
       <c r="H16" s="5"/>
       <c r="I16" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J16" s="5">
-        <v>10</v>
-      </c>
-      <c r="K16" s="7">
+        <v>15</v>
+      </c>
+      <c r="K16" s="8">
         <v>46113</v>
       </c>
       <c r="L16" s="4">
@@ -1503,19 +1410,15 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
-        <v>3200</v>
+        <v>2000</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="D17" s="5">
-        <v>18689</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
       <c r="E17" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F17" s="5">
         <v>2001</v>
@@ -1523,12 +1426,12 @@
       <c r="G17" s="5"/>
       <c r="H17" s="5"/>
       <c r="I17" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J17" s="5">
         <v>10</v>
       </c>
-      <c r="K17" s="7">
+      <c r="K17" s="8">
         <v>46113</v>
       </c>
       <c r="L17" s="4">
@@ -1537,19 +1440,16 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
-        <v>3200</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D18" s="5">
-        <v>18690</v>
-      </c>
+        <v>3600</v>
+      </c>
+      <c r="B18" s="5" t="str">
+        <f>TRIM(K19)</f>
+        <v>46113</v>
+      </c>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
       <c r="E18" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F18" s="5">
         <v>2001</v>
@@ -1557,12 +1457,12 @@
       <c r="G18" s="5"/>
       <c r="H18" s="5"/>
       <c r="I18" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J18" s="5">
-        <v>10</v>
-      </c>
-      <c r="K18" s="7">
+        <v>15</v>
+      </c>
+      <c r="K18" s="8">
         <v>46113</v>
       </c>
       <c r="L18" s="4">
@@ -1571,19 +1471,16 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
-        <v>3200</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D19" s="5">
-        <v>18691</v>
-      </c>
+        <v>3600</v>
+      </c>
+      <c r="B19" s="5" t="str">
+        <f>TRIM(K20)</f>
+        <v>46113</v>
+      </c>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
       <c r="E19" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F19" s="5">
         <v>2001</v>
@@ -1591,12 +1488,12 @@
       <c r="G19" s="5"/>
       <c r="H19" s="5"/>
       <c r="I19" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J19" s="5">
-        <v>10</v>
-      </c>
-      <c r="K19" s="7">
+        <v>15</v>
+      </c>
+      <c r="K19" s="8">
         <v>46113</v>
       </c>
       <c r="L19" s="4">
@@ -1605,15 +1502,16 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
-        <v>3200</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>34</v>
+        <v>3600</v>
+      </c>
+      <c r="B20" s="5" t="str">
+        <f>TRIM(K21)</f>
+        <v>46113</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
       <c r="E20" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F20" s="5">
         <v>2001</v>
@@ -1621,12 +1519,12 @@
       <c r="G20" s="5"/>
       <c r="H20" s="5"/>
       <c r="I20" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J20" s="5">
-        <v>10</v>
-      </c>
-      <c r="K20" s="7">
+        <v>15</v>
+      </c>
+      <c r="K20" s="8">
         <v>46113</v>
       </c>
       <c r="L20" s="4">
@@ -1635,15 +1533,15 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
       <c r="E21" s="5" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F21" s="5">
         <v>2001</v>
@@ -1651,12 +1549,12 @@
       <c r="G21" s="5"/>
       <c r="H21" s="5"/>
       <c r="I21" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J21" s="5">
-        <v>10</v>
-      </c>
-      <c r="K21" s="7">
+        <v>15</v>
+      </c>
+      <c r="K21" s="8">
         <v>46113</v>
       </c>
       <c r="L21" s="4">
@@ -1665,19 +1563,15 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D22" s="5">
-        <v>19039</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
       <c r="E22" s="5" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F22" s="5">
         <v>2001</v>
@@ -1685,12 +1579,12 @@
       <c r="G22" s="5"/>
       <c r="H22" s="5"/>
       <c r="I22" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J22" s="5">
-        <v>10</v>
-      </c>
-      <c r="K22" s="7">
+        <v>15</v>
+      </c>
+      <c r="K22" s="8">
         <v>46113</v>
       </c>
       <c r="L22" s="4">
@@ -1699,19 +1593,15 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="D23" s="5">
-        <v>19040</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
       <c r="E23" s="5" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F23" s="5">
         <v>2001</v>
@@ -1719,12 +1609,12 @@
       <c r="G23" s="5"/>
       <c r="H23" s="5"/>
       <c r="I23" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J23" s="5">
-        <v>10</v>
-      </c>
-      <c r="K23" s="7">
+        <v>15</v>
+      </c>
+      <c r="K23" s="8">
         <v>46113</v>
       </c>
       <c r="L23" s="4">
@@ -1733,15 +1623,15 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
       <c r="E24" s="5" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F24" s="5">
         <v>2001</v>
@@ -1749,12 +1639,12 @@
       <c r="G24" s="5"/>
       <c r="H24" s="5"/>
       <c r="I24" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J24" s="5">
-        <v>10</v>
-      </c>
-      <c r="K24" s="7">
+        <v>15</v>
+      </c>
+      <c r="K24" s="8">
         <v>46113</v>
       </c>
       <c r="L24" s="4">
@@ -1763,15 +1653,15 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
       <c r="E25" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F25" s="5">
         <v>2001</v>
@@ -1779,12 +1669,12 @@
       <c r="G25" s="5"/>
       <c r="H25" s="5"/>
       <c r="I25" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J25" s="5">
-        <v>10</v>
-      </c>
-      <c r="K25" s="7">
+        <v>15</v>
+      </c>
+      <c r="K25" s="8">
         <v>46113</v>
       </c>
       <c r="L25" s="4">
@@ -1793,15 +1683,15 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
       <c r="E26" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F26" s="5">
         <v>2001</v>
@@ -1809,12 +1699,12 @@
       <c r="G26" s="5"/>
       <c r="H26" s="5"/>
       <c r="I26" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J26" s="5">
-        <v>10</v>
-      </c>
-      <c r="K26" s="7">
+        <v>15</v>
+      </c>
+      <c r="K26" s="8">
         <v>46113</v>
       </c>
       <c r="L26" s="4">
@@ -1823,15 +1713,15 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
       <c r="E27" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F27" s="5">
         <v>2001</v>
@@ -1839,12 +1729,12 @@
       <c r="G27" s="5"/>
       <c r="H27" s="5"/>
       <c r="I27" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J27" s="5">
-        <v>10</v>
-      </c>
-      <c r="K27" s="7">
+        <v>15</v>
+      </c>
+      <c r="K27" s="8">
         <v>46113</v>
       </c>
       <c r="L27" s="4">
@@ -1853,15 +1743,15 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
       <c r="E28" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F28" s="5">
         <v>2001</v>
@@ -1869,12 +1759,12 @@
       <c r="G28" s="5"/>
       <c r="H28" s="5"/>
       <c r="I28" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J28" s="5">
-        <v>10</v>
-      </c>
-      <c r="K28" s="7">
+        <v>15</v>
+      </c>
+      <c r="K28" s="8">
         <v>46113</v>
       </c>
       <c r="L28" s="4">
@@ -1883,15 +1773,15 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="5"/>
       <c r="E29" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F29" s="5">
         <v>2001</v>
@@ -1899,12 +1789,12 @@
       <c r="G29" s="5"/>
       <c r="H29" s="5"/>
       <c r="I29" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J29" s="5">
-        <v>10</v>
-      </c>
-      <c r="K29" s="7">
+        <v>15</v>
+      </c>
+      <c r="K29" s="8">
         <v>46113</v>
       </c>
       <c r="L29" s="4">
@@ -1913,15 +1803,15 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="5"/>
       <c r="E30" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F30" s="5">
         <v>2001</v>
@@ -1929,12 +1819,12 @@
       <c r="G30" s="5"/>
       <c r="H30" s="5"/>
       <c r="I30" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J30" s="5">
-        <v>10</v>
-      </c>
-      <c r="K30" s="7">
+        <v>15</v>
+      </c>
+      <c r="K30" s="8">
         <v>46113</v>
       </c>
       <c r="L30" s="4">
@@ -1943,15 +1833,15 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="5"/>
       <c r="E31" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F31" s="5">
         <v>2001</v>
@@ -1959,12 +1849,12 @@
       <c r="G31" s="5"/>
       <c r="H31" s="5"/>
       <c r="I31" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J31" s="5">
-        <v>10</v>
-      </c>
-      <c r="K31" s="7">
+        <v>15</v>
+      </c>
+      <c r="K31" s="8">
         <v>46113</v>
       </c>
       <c r="L31" s="4">
@@ -1973,15 +1863,15 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="5"/>
       <c r="E32" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F32" s="5">
         <v>2001</v>
@@ -1989,12 +1879,12 @@
       <c r="G32" s="5"/>
       <c r="H32" s="5"/>
       <c r="I32" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J32" s="5">
-        <v>10</v>
-      </c>
-      <c r="K32" s="7">
+        <v>15</v>
+      </c>
+      <c r="K32" s="8">
         <v>46113</v>
       </c>
       <c r="L32" s="4">
@@ -2003,15 +1893,15 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="5"/>
       <c r="E33" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F33" s="5">
         <v>2001</v>
@@ -2019,12 +1909,12 @@
       <c r="G33" s="5"/>
       <c r="H33" s="5"/>
       <c r="I33" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J33" s="5">
-        <v>10</v>
-      </c>
-      <c r="K33" s="7">
+        <v>15</v>
+      </c>
+      <c r="K33" s="8">
         <v>46113</v>
       </c>
       <c r="L33" s="4">
@@ -2033,15 +1923,15 @@
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="5"/>
       <c r="E34" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F34" s="5">
         <v>2001</v>
@@ -2049,12 +1939,12 @@
       <c r="G34" s="5"/>
       <c r="H34" s="5"/>
       <c r="I34" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J34" s="5">
-        <v>10</v>
-      </c>
-      <c r="K34" s="7">
+        <v>15</v>
+      </c>
+      <c r="K34" s="8">
         <v>46113</v>
       </c>
       <c r="L34" s="4">
@@ -2063,15 +1953,15 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A35" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="C35" s="5"/>
       <c r="D35" s="5"/>
       <c r="E35" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F35" s="5">
         <v>2001</v>
@@ -2079,12 +1969,12 @@
       <c r="G35" s="5"/>
       <c r="H35" s="5"/>
       <c r="I35" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J35" s="5">
-        <v>10</v>
-      </c>
-      <c r="K35" s="7">
+        <v>15</v>
+      </c>
+      <c r="K35" s="8">
         <v>46113</v>
       </c>
       <c r="L35" s="4">
@@ -2093,15 +1983,15 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A36" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="5"/>
       <c r="E36" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F36" s="5">
         <v>2001</v>
@@ -2109,12 +1999,12 @@
       <c r="G36" s="5"/>
       <c r="H36" s="5"/>
       <c r="I36" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J36" s="5">
-        <v>10</v>
-      </c>
-      <c r="K36" s="7">
+        <v>15</v>
+      </c>
+      <c r="K36" s="8">
         <v>46113</v>
       </c>
       <c r="L36" s="4">
@@ -2123,15 +2013,15 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A37" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="C37" s="5"/>
       <c r="D37" s="5"/>
       <c r="E37" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F37" s="5">
         <v>2001</v>
@@ -2139,12 +2029,12 @@
       <c r="G37" s="5"/>
       <c r="H37" s="5"/>
       <c r="I37" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J37" s="5">
-        <v>10</v>
-      </c>
-      <c r="K37" s="7">
+        <v>15</v>
+      </c>
+      <c r="K37" s="8">
         <v>46113</v>
       </c>
       <c r="L37" s="4">
@@ -2153,15 +2043,15 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A38" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" s="5"/>
       <c r="E38" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F38" s="5">
         <v>2001</v>
@@ -2169,12 +2059,12 @@
       <c r="G38" s="5"/>
       <c r="H38" s="5"/>
       <c r="I38" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J38" s="5">
-        <v>10</v>
-      </c>
-      <c r="K38" s="7">
+        <v>15</v>
+      </c>
+      <c r="K38" s="8">
         <v>46113</v>
       </c>
       <c r="L38" s="4">
@@ -2183,15 +2073,15 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A39" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5"/>
       <c r="E39" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F39" s="5">
         <v>2001</v>
@@ -2199,12 +2089,12 @@
       <c r="G39" s="5"/>
       <c r="H39" s="5"/>
       <c r="I39" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J39" s="5">
-        <v>10</v>
-      </c>
-      <c r="K39" s="7">
+        <v>15</v>
+      </c>
+      <c r="K39" s="8">
         <v>46113</v>
       </c>
       <c r="L39" s="4">
@@ -2213,15 +2103,15 @@
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A40" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="C40" s="5"/>
       <c r="D40" s="5"/>
       <c r="E40" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F40" s="5">
         <v>2001</v>
@@ -2229,12 +2119,12 @@
       <c r="G40" s="5"/>
       <c r="H40" s="5"/>
       <c r="I40" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J40" s="5">
-        <v>10</v>
-      </c>
-      <c r="K40" s="7">
+        <v>15</v>
+      </c>
+      <c r="K40" s="8">
         <v>46113</v>
       </c>
       <c r="L40" s="4">
@@ -2243,15 +2133,15 @@
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A41" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
       <c r="E41" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F41" s="5">
         <v>2001</v>
@@ -2259,12 +2149,12 @@
       <c r="G41" s="5"/>
       <c r="H41" s="5"/>
       <c r="I41" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J41" s="5">
-        <v>10</v>
-      </c>
-      <c r="K41" s="7">
+        <v>15</v>
+      </c>
+      <c r="K41" s="8">
         <v>46113</v>
       </c>
       <c r="L41" s="4">
@@ -2273,15 +2163,15 @@
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A42" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="C42" s="5"/>
       <c r="D42" s="5"/>
       <c r="E42" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F42" s="5">
         <v>2001</v>
@@ -2289,12 +2179,12 @@
       <c r="G42" s="5"/>
       <c r="H42" s="5"/>
       <c r="I42" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J42" s="5">
-        <v>10</v>
-      </c>
-      <c r="K42" s="7">
+        <v>15</v>
+      </c>
+      <c r="K42" s="8">
         <v>46113</v>
       </c>
       <c r="L42" s="4">
@@ -2303,15 +2193,15 @@
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A43" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="5"/>
       <c r="E43" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F43" s="5">
         <v>2001</v>
@@ -2319,12 +2209,12 @@
       <c r="G43" s="5"/>
       <c r="H43" s="5"/>
       <c r="I43" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J43" s="5">
-        <v>10</v>
-      </c>
-      <c r="K43" s="7">
+        <v>15</v>
+      </c>
+      <c r="K43" s="8">
         <v>46113</v>
       </c>
       <c r="L43" s="4">
@@ -2333,15 +2223,15 @@
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A44" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="C44" s="5"/>
       <c r="D44" s="5"/>
       <c r="E44" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F44" s="5">
         <v>2001</v>
@@ -2349,12 +2239,12 @@
       <c r="G44" s="5"/>
       <c r="H44" s="5"/>
       <c r="I44" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J44" s="5">
-        <v>10</v>
-      </c>
-      <c r="K44" s="7">
+        <v>15</v>
+      </c>
+      <c r="K44" s="8">
         <v>46113</v>
       </c>
       <c r="L44" s="4">
@@ -2363,15 +2253,15 @@
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A45" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5"/>
       <c r="E45" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F45" s="5">
         <v>2001</v>
@@ -2379,12 +2269,12 @@
       <c r="G45" s="5"/>
       <c r="H45" s="5"/>
       <c r="I45" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J45" s="5">
-        <v>10</v>
-      </c>
-      <c r="K45" s="7">
+        <v>15</v>
+      </c>
+      <c r="K45" s="8">
         <v>46113</v>
       </c>
       <c r="L45" s="4">
@@ -2393,15 +2283,15 @@
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A46" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C46" s="5"/>
       <c r="D46" s="5"/>
       <c r="E46" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F46" s="5">
         <v>2001</v>
@@ -2409,12 +2299,12 @@
       <c r="G46" s="5"/>
       <c r="H46" s="5"/>
       <c r="I46" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J46" s="5">
-        <v>10</v>
-      </c>
-      <c r="K46" s="7">
+        <v>15</v>
+      </c>
+      <c r="K46" s="8">
         <v>46113</v>
       </c>
       <c r="L46" s="4">
@@ -2423,15 +2313,15 @@
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A47" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C47" s="5"/>
       <c r="D47" s="5"/>
       <c r="E47" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F47" s="5">
         <v>2001</v>
@@ -2439,12 +2329,12 @@
       <c r="G47" s="5"/>
       <c r="H47" s="5"/>
       <c r="I47" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J47" s="5">
-        <v>10</v>
-      </c>
-      <c r="K47" s="7">
+        <v>15</v>
+      </c>
+      <c r="K47" s="8">
         <v>46113</v>
       </c>
       <c r="L47" s="4">
@@ -2453,15 +2343,15 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A48" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C48" s="5"/>
       <c r="D48" s="5"/>
       <c r="E48" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F48" s="5">
         <v>2001</v>
@@ -2469,12 +2359,12 @@
       <c r="G48" s="5"/>
       <c r="H48" s="5"/>
       <c r="I48" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J48" s="5">
-        <v>10</v>
-      </c>
-      <c r="K48" s="7">
+        <v>15</v>
+      </c>
+      <c r="K48" s="8">
         <v>46113</v>
       </c>
       <c r="L48" s="4">
@@ -2483,15 +2373,15 @@
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A49" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C49" s="5"/>
       <c r="D49" s="5"/>
       <c r="E49" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F49" s="5">
         <v>2001</v>
@@ -2499,12 +2389,12 @@
       <c r="G49" s="5"/>
       <c r="H49" s="5"/>
       <c r="I49" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J49" s="5">
-        <v>10</v>
-      </c>
-      <c r="K49" s="7">
+        <v>15</v>
+      </c>
+      <c r="K49" s="8">
         <v>46113</v>
       </c>
       <c r="L49" s="4">
@@ -2513,15 +2403,15 @@
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A50" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C50" s="5"/>
       <c r="D50" s="5"/>
       <c r="E50" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F50" s="5">
         <v>2001</v>
@@ -2529,12 +2419,12 @@
       <c r="G50" s="5"/>
       <c r="H50" s="5"/>
       <c r="I50" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J50" s="5">
-        <v>10</v>
-      </c>
-      <c r="K50" s="7">
+        <v>15</v>
+      </c>
+      <c r="K50" s="8">
         <v>46113</v>
       </c>
       <c r="L50" s="4">
@@ -2543,15 +2433,15 @@
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A51" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="C51" s="5"/>
       <c r="D51" s="5"/>
       <c r="E51" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F51" s="5">
         <v>2001</v>
@@ -2559,12 +2449,12 @@
       <c r="G51" s="5"/>
       <c r="H51" s="5"/>
       <c r="I51" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J51" s="5">
-        <v>10</v>
-      </c>
-      <c r="K51" s="7">
+        <v>15</v>
+      </c>
+      <c r="K51" s="8">
         <v>46113</v>
       </c>
       <c r="L51" s="4">
@@ -2573,15 +2463,15 @@
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A52" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="C52" s="5"/>
       <c r="D52" s="5"/>
       <c r="E52" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F52" s="5">
         <v>2001</v>
@@ -2589,12 +2479,12 @@
       <c r="G52" s="5"/>
       <c r="H52" s="5"/>
       <c r="I52" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J52" s="5">
-        <v>10</v>
-      </c>
-      <c r="K52" s="7">
+        <v>15</v>
+      </c>
+      <c r="K52" s="8">
         <v>46113</v>
       </c>
       <c r="L52" s="4">
@@ -2603,15 +2493,15 @@
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A53" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="5"/>
       <c r="E53" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F53" s="5">
         <v>2001</v>
@@ -2619,12 +2509,12 @@
       <c r="G53" s="5"/>
       <c r="H53" s="5"/>
       <c r="I53" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J53" s="5">
-        <v>10</v>
-      </c>
-      <c r="K53" s="7">
+        <v>15</v>
+      </c>
+      <c r="K53" s="8">
         <v>46113</v>
       </c>
       <c r="L53" s="4">
@@ -2633,15 +2523,15 @@
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A54" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="C54" s="5"/>
       <c r="D54" s="5"/>
       <c r="E54" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F54" s="5">
         <v>2001</v>
@@ -2649,12 +2539,12 @@
       <c r="G54" s="5"/>
       <c r="H54" s="5"/>
       <c r="I54" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J54" s="5">
-        <v>10</v>
-      </c>
-      <c r="K54" s="7">
+        <v>15</v>
+      </c>
+      <c r="K54" s="8">
         <v>46113</v>
       </c>
       <c r="L54" s="4">
@@ -2663,15 +2553,15 @@
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A55" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="C55" s="5"/>
       <c r="D55" s="5"/>
       <c r="E55" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F55" s="5">
         <v>2001</v>
@@ -2679,12 +2569,12 @@
       <c r="G55" s="5"/>
       <c r="H55" s="5"/>
       <c r="I55" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J55" s="5">
-        <v>10</v>
-      </c>
-      <c r="K55" s="7">
+        <v>15</v>
+      </c>
+      <c r="K55" s="8">
         <v>46113</v>
       </c>
       <c r="L55" s="4">
@@ -2693,15 +2583,15 @@
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A56" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="C56" s="5"/>
       <c r="D56" s="5"/>
       <c r="E56" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F56" s="5">
         <v>2001</v>
@@ -2709,12 +2599,12 @@
       <c r="G56" s="5"/>
       <c r="H56" s="5"/>
       <c r="I56" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J56" s="5">
-        <v>10</v>
-      </c>
-      <c r="K56" s="7">
+        <v>15</v>
+      </c>
+      <c r="K56" s="8">
         <v>46113</v>
       </c>
       <c r="L56" s="4">
@@ -2723,15 +2613,15 @@
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A57" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="C57" s="5"/>
       <c r="D57" s="5"/>
       <c r="E57" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F57" s="5">
         <v>2001</v>
@@ -2739,12 +2629,12 @@
       <c r="G57" s="5"/>
       <c r="H57" s="5"/>
       <c r="I57" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J57" s="5">
-        <v>10</v>
-      </c>
-      <c r="K57" s="7">
+        <v>15</v>
+      </c>
+      <c r="K57" s="8">
         <v>46113</v>
       </c>
       <c r="L57" s="4">
@@ -2753,15 +2643,15 @@
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A58" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="5"/>
       <c r="E58" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F58" s="5">
         <v>2001</v>
@@ -2769,12 +2659,12 @@
       <c r="G58" s="5"/>
       <c r="H58" s="5"/>
       <c r="I58" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J58" s="5">
-        <v>10</v>
-      </c>
-      <c r="K58" s="7">
+        <v>15</v>
+      </c>
+      <c r="K58" s="8">
         <v>46113</v>
       </c>
       <c r="L58" s="4">
@@ -2783,15 +2673,15 @@
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A59" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="C59" s="5"/>
       <c r="D59" s="5"/>
       <c r="E59" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F59" s="5">
         <v>2001</v>
@@ -2799,12 +2689,12 @@
       <c r="G59" s="5"/>
       <c r="H59" s="5"/>
       <c r="I59" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J59" s="5">
-        <v>10</v>
-      </c>
-      <c r="K59" s="7">
+        <v>15</v>
+      </c>
+      <c r="K59" s="8">
         <v>46113</v>
       </c>
       <c r="L59" s="4">
@@ -2813,15 +2703,15 @@
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A60" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C60" s="5"/>
       <c r="D60" s="5"/>
       <c r="E60" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F60" s="5">
         <v>2001</v>
@@ -2829,12 +2719,12 @@
       <c r="G60" s="5"/>
       <c r="H60" s="5"/>
       <c r="I60" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J60" s="5">
-        <v>10</v>
-      </c>
-      <c r="K60" s="7">
+        <v>15</v>
+      </c>
+      <c r="K60" s="8">
         <v>46113</v>
       </c>
       <c r="L60" s="4">
@@ -2843,15 +2733,15 @@
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A61" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C61" s="5"/>
       <c r="D61" s="5"/>
       <c r="E61" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F61" s="5">
         <v>2001</v>
@@ -2859,12 +2749,12 @@
       <c r="G61" s="5"/>
       <c r="H61" s="5"/>
       <c r="I61" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J61" s="5">
-        <v>10</v>
-      </c>
-      <c r="K61" s="7">
+        <v>15</v>
+      </c>
+      <c r="K61" s="8">
         <v>46113</v>
       </c>
       <c r="L61" s="4">
@@ -2873,15 +2763,15 @@
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A62" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="C62" s="5"/>
       <c r="D62" s="5"/>
       <c r="E62" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F62" s="5">
         <v>2001</v>
@@ -2889,12 +2779,12 @@
       <c r="G62" s="5"/>
       <c r="H62" s="5"/>
       <c r="I62" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J62" s="5">
-        <v>10</v>
-      </c>
-      <c r="K62" s="7">
+        <v>15</v>
+      </c>
+      <c r="K62" s="8">
         <v>46113</v>
       </c>
       <c r="L62" s="4">
@@ -2903,15 +2793,15 @@
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A63" s="5">
-        <v>3200</v>
+        <v>3600</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="C63" s="5"/>
       <c r="D63" s="5"/>
       <c r="E63" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F63" s="5">
         <v>2001</v>
@@ -2919,15 +2809,75 @@
       <c r="G63" s="5"/>
       <c r="H63" s="5"/>
       <c r="I63" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="J63" s="5">
-        <v>10</v>
-      </c>
-      <c r="K63" s="7">
+        <v>15</v>
+      </c>
+      <c r="K63" s="8">
         <v>46113</v>
       </c>
       <c r="L63" s="4">
+        <v>46113</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A64" s="5">
+        <v>3600</v>
+      </c>
+      <c r="B64" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C64" s="7"/>
+      <c r="D64" s="7"/>
+      <c r="E64" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F64" s="5">
+        <v>2001</v>
+      </c>
+      <c r="G64" s="6"/>
+      <c r="H64" s="6"/>
+      <c r="I64" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J64" s="5">
+        <v>15</v>
+      </c>
+      <c r="K64" s="8">
+        <v>46113</v>
+      </c>
+      <c r="L64" s="4">
+        <v>46113</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A65" s="5">
+        <v>3600</v>
+      </c>
+      <c r="B65" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C65" s="7"/>
+      <c r="D65" s="7"/>
+      <c r="E65" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F65" s="5">
+        <v>2001</v>
+      </c>
+      <c r="G65" s="6"/>
+      <c r="H65" s="6"/>
+      <c r="I65" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J65" s="5">
+        <v>15</v>
+      </c>
+      <c r="K65" s="8">
+        <v>46113</v>
+      </c>
+      <c r="L65" s="4">
         <v>46113</v>
       </c>
     </row>
@@ -2941,6 +2891,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4e5a10fa-5ff6-486e-a842-9b38fcf2e5f3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EB579093A7D6834CB4AC0F2FEE371DF1" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b7a0b863fc9807cbcab59f944e049a35">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4e5a10fa-5ff6-486e-a842-9b38fcf2e5f3" xmlns:ns3="1112ab2c-f21c-4197-be07-89a75d2423ba" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="97c90fb0047f9bad8e219a244397e680" ns2:_="" ns3:_="">
     <xsd:import namespace="4e5a10fa-5ff6-486e-a842-9b38fcf2e5f3"/>
@@ -3169,40 +3138,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4e5a10fa-5ff6-486e-a842-9b38fcf2e5f3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0632B208-E20D-4AC6-92D8-02837DA03E16}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F1D4C1C-B842-42FF-A3CF-55D898A8C96F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="4e5a10fa-5ff6-486e-a842-9b38fcf2e5f3"/>
-    <ds:schemaRef ds:uri="1112ab2c-f21c-4197-be07-89a75d2423ba"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3225,9 +3164,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F1D4C1C-B842-42FF-A3CF-55D898A8C96F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0632B208-E20D-4AC6-92D8-02837DA03E16}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="4e5a10fa-5ff6-486e-a842-9b38fcf2e5f3"/>
+    <ds:schemaRef ds:uri="1112ab2c-f21c-4197-be07-89a75d2423ba"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>